<commit_message>
Actualiza elmo_data.xlsx para escenario Swap_max_production_160kW
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Taller_DET_Agosto/Swap_max_production_160kW/elmo_data.xlsx
+++ b/data/Taller_DET_Agosto/Swap_max_production_160kW/elmo_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Agustin\Desktop\Elmo_infrastructure_NP\data\Taller_DET_Agosto\Swap_max_production_160kW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\Taller_DET_Agosto\Swap_max_production_160kW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0567F972-AB08-490E-84F2-314EB77D2144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CA7C4C-13E3-4E7E-99E7-5F7B188702B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LHD" sheetId="2" r:id="rId1"/>
@@ -1493,38 +1493,38 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:AD9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.33203125" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.44140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="5" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="15" style="5" customWidth="1"/>
-    <col min="16" max="16" width="16.88671875" style="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="18" style="6" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="20.88671875" style="6" bestFit="1" customWidth="1"/>
-    <col min="20" max="23" width="20.88671875" style="6" customWidth="1"/>
-    <col min="24" max="24" width="18.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="20.109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.33203125" style="6" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="19.109375" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="20.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="20.85546875" style="6" customWidth="1"/>
+    <col min="24" max="24" width="18.42578125" style="6" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="20.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="8.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -1984,7 +1984,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2076,7 +2076,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2362,16 +2362,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC93900-5A86-4519-AB89-460E8AC441EE}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -2449,8 +2449,8 @@
         <v>59</v>
       </c>
       <c r="C3" s="8">
-        <f>2*35722</f>
-        <v>71444</v>
+        <f>35722</f>
+        <v>35722</v>
       </c>
       <c r="D3" s="14">
         <v>38221</v>
@@ -2465,7 +2465,7 @@
         <v>4389</v>
       </c>
       <c r="H3" s="15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3" s="15">
         <v>2</v>
@@ -2474,7 +2474,7 @@
         <v>2</v>
       </c>
       <c r="K3" s="8">
-        <v>2400</v>
+        <v>1200</v>
       </c>
     </row>
   </sheetData>
@@ -2486,14 +2486,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5C58D2-31A1-4CA6-99E5-3102447D41CF}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2519,7 +2519,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -2582,17 +2582,17 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H236"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -2618,7 +2618,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -2644,7 +2644,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -2670,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -2696,7 +2696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -2852,7 +2852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -2904,7 +2904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2930,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -2956,7 +2956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>14</v>
       </c>
@@ -3008,7 +3008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>15</v>
       </c>
@@ -3034,7 +3034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>16</v>
       </c>
@@ -3060,7 +3060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>17</v>
       </c>
@@ -3086,7 +3086,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>18</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>19</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>20</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>21</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>22</v>
       </c>
@@ -3216,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>23</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24</v>
       </c>
@@ -3268,7 +3268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>25</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>26</v>
       </c>
@@ -3320,7 +3320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>27</v>
       </c>
@@ -3346,7 +3346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>28</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>29</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30</v>
       </c>
@@ -3424,7 +3424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>31</v>
       </c>
@@ -3450,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>32</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>33</v>
       </c>
@@ -3502,7 +3502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>34</v>
       </c>
@@ -3528,7 +3528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>35</v>
       </c>
@@ -3554,7 +3554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>36</v>
       </c>
@@ -3580,7 +3580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>37</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>38</v>
       </c>
@@ -3632,7 +3632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>39</v>
       </c>
@@ -3658,7 +3658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>40</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>41</v>
       </c>
@@ -3710,7 +3710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>42</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>43</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>44</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>45</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>46</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>47</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>48</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>49</v>
       </c>
@@ -3918,7 +3918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>50</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>51</v>
       </c>
@@ -3970,7 +3970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>52</v>
       </c>
@@ -3996,7 +3996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>53</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>54</v>
       </c>
@@ -4048,7 +4048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>55</v>
       </c>
@@ -4074,7 +4074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>56</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>57</v>
       </c>
@@ -4126,7 +4126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>58</v>
       </c>
@@ -4152,7 +4152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>59</v>
       </c>
@@ -4178,7 +4178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>60</v>
       </c>
@@ -4204,7 +4204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>61</v>
       </c>
@@ -4230,7 +4230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>62</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>63</v>
       </c>
@@ -4282,7 +4282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>64</v>
       </c>
@@ -4308,7 +4308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>65</v>
       </c>
@@ -4334,7 +4334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>66</v>
       </c>
@@ -4360,7 +4360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>67</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>68</v>
       </c>
@@ -4412,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>69</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>70</v>
       </c>
@@ -4464,7 +4464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>71</v>
       </c>
@@ -4490,7 +4490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>72</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>73</v>
       </c>
@@ -4542,7 +4542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>74</v>
       </c>
@@ -4568,7 +4568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>75</v>
       </c>
@@ -4594,7 +4594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>76</v>
       </c>
@@ -4620,7 +4620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>77</v>
       </c>
@@ -4646,7 +4646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>78</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>79</v>
       </c>
@@ -4698,7 +4698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>80</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>81</v>
       </c>
@@ -4750,7 +4750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>82</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>83</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>84</v>
       </c>
@@ -4828,7 +4828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>85</v>
       </c>
@@ -4854,7 +4854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>86</v>
       </c>
@@ -4880,7 +4880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>87</v>
       </c>
@@ -4906,7 +4906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>88</v>
       </c>
@@ -4932,7 +4932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>89</v>
       </c>
@@ -4958,7 +4958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>90</v>
       </c>
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>91</v>
       </c>
@@ -5010,7 +5010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>92</v>
       </c>
@@ -5036,7 +5036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>93</v>
       </c>
@@ -5062,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>94</v>
       </c>
@@ -5088,7 +5088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>95</v>
       </c>
@@ -5114,7 +5114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>96</v>
       </c>
@@ -5140,7 +5140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>97</v>
       </c>
@@ -5166,7 +5166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>98</v>
       </c>
@@ -5192,7 +5192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>99</v>
       </c>
@@ -5218,7 +5218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>100</v>
       </c>
@@ -5244,7 +5244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>101</v>
       </c>
@@ -5270,7 +5270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>102</v>
       </c>
@@ -5296,7 +5296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>103</v>
       </c>
@@ -5322,7 +5322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>104</v>
       </c>
@@ -5348,7 +5348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>105</v>
       </c>
@@ -5374,7 +5374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>106</v>
       </c>
@@ -5400,7 +5400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>107</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>108</v>
       </c>
@@ -5452,7 +5452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>109</v>
       </c>
@@ -5478,7 +5478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>110</v>
       </c>
@@ -5504,7 +5504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>111</v>
       </c>
@@ -5530,7 +5530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>112</v>
       </c>
@@ -5556,7 +5556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>113</v>
       </c>
@@ -5582,7 +5582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>114</v>
       </c>
@@ -5608,7 +5608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>115</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>116</v>
       </c>
@@ -5660,7 +5660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>117</v>
       </c>
@@ -5686,7 +5686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>118</v>
       </c>
@@ -5712,7 +5712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>119</v>
       </c>
@@ -5738,7 +5738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>120</v>
       </c>
@@ -5764,7 +5764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>121</v>
       </c>
@@ -5790,7 +5790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>122</v>
       </c>
@@ -5816,7 +5816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>123</v>
       </c>
@@ -5842,7 +5842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>124</v>
       </c>
@@ -5868,7 +5868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>125</v>
       </c>
@@ -5894,7 +5894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>126</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>127</v>
       </c>
@@ -5946,7 +5946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>128</v>
       </c>
@@ -5972,7 +5972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>129</v>
       </c>
@@ -5998,7 +5998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>130</v>
       </c>
@@ -6024,7 +6024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>131</v>
       </c>
@@ -6050,7 +6050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>132</v>
       </c>
@@ -6076,7 +6076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>133</v>
       </c>
@@ -6102,7 +6102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>134</v>
       </c>
@@ -6128,7 +6128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>135</v>
       </c>
@@ -6154,7 +6154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>136</v>
       </c>
@@ -6180,7 +6180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>137</v>
       </c>
@@ -6206,7 +6206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>138</v>
       </c>
@@ -6232,7 +6232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>139</v>
       </c>
@@ -6258,7 +6258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>140</v>
       </c>
@@ -6284,7 +6284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>141</v>
       </c>
@@ -6310,7 +6310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>142</v>
       </c>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>143</v>
       </c>
@@ -6362,7 +6362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>144</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>145</v>
       </c>
@@ -6414,7 +6414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>146</v>
       </c>
@@ -6440,7 +6440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>147</v>
       </c>
@@ -6466,7 +6466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>148</v>
       </c>
@@ -6492,7 +6492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>149</v>
       </c>
@@ -6518,7 +6518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>150</v>
       </c>
@@ -6544,7 +6544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>151</v>
       </c>
@@ -6570,7 +6570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>152</v>
       </c>
@@ -6596,7 +6596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>153</v>
       </c>
@@ -6622,7 +6622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>154</v>
       </c>
@@ -6648,7 +6648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>155</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>156</v>
       </c>
@@ -6700,7 +6700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>157</v>
       </c>
@@ -6726,7 +6726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>158</v>
       </c>
@@ -6752,7 +6752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>159</v>
       </c>
@@ -6778,7 +6778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>160</v>
       </c>
@@ -6804,7 +6804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>161</v>
       </c>
@@ -6830,7 +6830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>162</v>
       </c>
@@ -6856,7 +6856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>163</v>
       </c>
@@ -6882,7 +6882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>164</v>
       </c>
@@ -6908,7 +6908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>165</v>
       </c>
@@ -6934,7 +6934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>166</v>
       </c>
@@ -6960,7 +6960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>167</v>
       </c>
@@ -6986,7 +6986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>168</v>
       </c>
@@ -7012,7 +7012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>169</v>
       </c>
@@ -7038,7 +7038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>170</v>
       </c>
@@ -7064,7 +7064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>171</v>
       </c>
@@ -7090,7 +7090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>172</v>
       </c>
@@ -7116,7 +7116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>173</v>
       </c>
@@ -7142,7 +7142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>174</v>
       </c>
@@ -7168,7 +7168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>175</v>
       </c>
@@ -7194,7 +7194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>176</v>
       </c>
@@ -7220,7 +7220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>177</v>
       </c>
@@ -7246,7 +7246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>178</v>
       </c>
@@ -7272,7 +7272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>179</v>
       </c>
@@ -7298,7 +7298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>180</v>
       </c>
@@ -7324,7 +7324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>181</v>
       </c>
@@ -7350,7 +7350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>182</v>
       </c>
@@ -7376,7 +7376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>183</v>
       </c>
@@ -7402,7 +7402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>184</v>
       </c>
@@ -7428,7 +7428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>185</v>
       </c>
@@ -7454,7 +7454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>186</v>
       </c>
@@ -7480,7 +7480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>187</v>
       </c>
@@ -7506,7 +7506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>188</v>
       </c>
@@ -7532,7 +7532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>189</v>
       </c>
@@ -7558,7 +7558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>190</v>
       </c>
@@ -7584,7 +7584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>191</v>
       </c>
@@ -7610,7 +7610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>192</v>
       </c>
@@ -7636,7 +7636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>193</v>
       </c>
@@ -7662,7 +7662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>194</v>
       </c>
@@ -7688,7 +7688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>195</v>
       </c>
@@ -7714,7 +7714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>196</v>
       </c>
@@ -7740,7 +7740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>197</v>
       </c>
@@ -7766,7 +7766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>198</v>
       </c>
@@ -7792,7 +7792,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>199</v>
       </c>
@@ -7818,7 +7818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>200</v>
       </c>
@@ -7844,7 +7844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>201</v>
       </c>
@@ -7870,7 +7870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>202</v>
       </c>
@@ -7896,7 +7896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>203</v>
       </c>
@@ -7922,7 +7922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>204</v>
       </c>
@@ -7948,7 +7948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>205</v>
       </c>
@@ -7974,7 +7974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>206</v>
       </c>
@@ -8000,7 +8000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>207</v>
       </c>
@@ -8026,7 +8026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>208</v>
       </c>
@@ -8052,7 +8052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>209</v>
       </c>
@@ -8078,7 +8078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>210</v>
       </c>
@@ -8104,90 +8104,90 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213"/>
       <c r="C213"/>
       <c r="D213"/>
       <c r="G213"/>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214"/>
       <c r="C214"/>
       <c r="D214"/>
       <c r="G214"/>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215"/>
       <c r="C215"/>
       <c r="D215"/>
       <c r="G215"/>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216"/>
       <c r="C216"/>
       <c r="D216"/>
       <c r="G216"/>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217"/>
       <c r="C217"/>
       <c r="D217"/>
       <c r="G217"/>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218"/>
       <c r="C218"/>
       <c r="D218"/>
       <c r="G218"/>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219"/>
       <c r="C219"/>
       <c r="D219"/>
       <c r="G219"/>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220"/>
       <c r="C220"/>
       <c r="D220"/>
       <c r="G220"/>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221"/>
       <c r="C221"/>
       <c r="D221"/>
       <c r="G221"/>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222"/>
       <c r="C222"/>
       <c r="D222"/>
       <c r="G222"/>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223"/>
       <c r="C223"/>
       <c r="D223"/>
       <c r="G223"/>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224"/>
       <c r="C224"/>
       <c r="D224"/>
       <c r="G224"/>
     </row>
-    <row r="225" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="226" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="227" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="228" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="229" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="230" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="231" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="232" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="233" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="234" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="235" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="236" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="225" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="226" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="227" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="228" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="229" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="230" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="231" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="232" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="233" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="234" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="235" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="236" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8200,14 +8200,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:C12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -8218,7 +8218,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -8229,7 +8229,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8240,7 +8240,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -8251,7 +8251,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -8262,7 +8262,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8273,7 +8273,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -8284,7 +8284,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>11</v>
       </c>
@@ -8295,7 +8295,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>12</v>
       </c>
@@ -8306,7 +8306,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>14</v>
       </c>
@@ -8317,7 +8317,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>15</v>
       </c>
@@ -8328,7 +8328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>16</v>
       </c>

</xml_diff>